<commit_message>
feat: show resume images and full Excel tables inline with automatic regeneration
</commit_message>
<xml_diff>
--- a/assets/documents/Yiqing_Tu_Performance.xlsx
+++ b/assets/documents/Yiqing_Tu_Performance.xlsx
@@ -112,7 +112,7 @@
     <t xml:space="preserve">outdcloset21 </t>
   </si>
   <si>
-    <t>195.5K</t>
+    <t>195.6K</t>
   </si>
   <si>
     <t>https://www.anystories.app/book/the-evil-alpha-marked-me/6863b47ee07e05a1778caf75</t>
@@ -136,7 +136,7 @@
     <t>Lola Pamola</t>
   </si>
   <si>
-    <t>103.1K</t>
+    <t>104.4K</t>
   </si>
   <si>
     <t>https://www.anystories.app/book/the-volkov-legacy/68b098388c7d08441837fcaf</t>

</xml_diff>